<commit_message>
docs: re-verify SharePoint governance controls
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/sharepoint-admin-checklist.xlsx
+++ b/assessment/templates/sharepoint-admin-checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SharePoint Admin" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SharePoint Admin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SharePoint Admin'!$A$4:$I$14</definedName>
@@ -637,7 +637,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>DSPM for AI oversharing assessment report (PDF/JSON export); Remediation backlog ticket count + closure cadence; Item-level remediation log entries for the last 30 days; List of sites with EEEU/Everyone sharing flagged + dispositioned</t>
+          <t>DSPM data risk assessment or oversharing assessment export (Excel/CSV/JSON/TSV); Remediation backlog ticket count + closure cadence; Item-level remediation log entries for the last 30 days; List of sites with EEEU/Everyone sharing flagged + dispositioned</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>PowerShell output showing Get-SPOTenantRestrictedSearchMode returns Enabled; Current allow-list site URLs (≤100) with business owner per site; RCD exception register for targeted site-level exclusions; Documented exit plan / transition target date to long-term Purview+SAM governance</t>
+          <t>Current RCD site list or tenant report with site justification, owner, and review date; If RSS was enabled before July 31, 2026: current allow-list site URLs (≤100) with business owner per site; Documented exit plan / transition target date to long-term Purview+SAM governance</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Pages sharing policy configuration; Sensitivity label enforcement for Pages content; External sharing restriction evidence; Sharing activity audit log entries for Pages</t>
+          <t>Cloud Policy scope for Create and view Copilot Pages and Copilot Notebooks plus code-preview setting; Sensitivity label enforcement for Pages content; External sharing restriction evidence for the supporting SharePoint and Loop collaboration surfaces; Sharing activity audit log entries for Pages</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>

</xml_diff>